<commit_message>
upload: month_plan for 2025-11-05 (051125/Monthly_Plan.xlsx)
</commit_message>
<xml_diff>
--- a/outputs/2025-11-05/inputs/month_plan.xlsx
+++ b/outputs/2025-11-05/inputs/month_plan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Flight Operations\Crew Sched and BD Shared Folder\2025\November\Input Files\Mu sigma\051125\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Flight Operations\Crew Sched and BD Shared Folder\2025\November\Input Files\KTree\051125\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8E7F0A7-37DA-4CB4-BB7E-27DA9CD81E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0B10B28-315E-4482-BEB5-616A881E27FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3283,7 +3283,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:E457"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
@@ -3312,7 +3311,7 @@
         <v>45967</v>
       </c>
     </row>
-    <row r="2" spans="1:5" hidden="1">
+    <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -3329,7 +3328,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" hidden="1">
+    <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -3346,7 +3345,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="4" spans="1:5" hidden="1">
+    <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -3363,7 +3362,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" hidden="1">
+    <row r="5" spans="1:5">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -3380,7 +3379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1">
+    <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
@@ -3397,7 +3396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1">
+    <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
@@ -3414,7 +3413,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1">
+    <row r="8" spans="1:5">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
@@ -3431,7 +3430,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" hidden="1">
+    <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -3448,7 +3447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1">
+    <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
@@ -3465,7 +3464,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1">
+    <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
@@ -3482,7 +3481,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1">
+    <row r="12" spans="1:5">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
@@ -3499,7 +3498,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" hidden="1">
+    <row r="13" spans="1:5">
       <c r="A13" s="1" t="s">
         <v>23</v>
       </c>
@@ -3516,7 +3515,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="14" spans="1:5" hidden="1">
+    <row r="14" spans="1:5">
       <c r="A14" s="1" t="s">
         <v>25</v>
       </c>
@@ -3533,7 +3532,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" hidden="1">
+    <row r="15" spans="1:5">
       <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
@@ -3550,7 +3549,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1">
+    <row r="16" spans="1:5">
       <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
@@ -3567,7 +3566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1">
+    <row r="17" spans="1:5">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
@@ -3584,7 +3583,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:5" hidden="1">
+    <row r="18" spans="1:5">
       <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
@@ -3601,7 +3600,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" hidden="1">
+    <row r="19" spans="1:5">
       <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
@@ -3618,7 +3617,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" hidden="1">
+    <row r="20" spans="1:5">
       <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
@@ -3635,7 +3634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1">
+    <row r="21" spans="1:5">
       <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
@@ -3652,7 +3651,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1">
+    <row r="22" spans="1:5">
       <c r="A22" s="1" t="s">
         <v>43</v>
       </c>
@@ -3669,7 +3668,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1">
+    <row r="23" spans="1:5">
       <c r="A23" s="1" t="s">
         <v>45</v>
       </c>
@@ -3686,7 +3685,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:5" hidden="1">
+    <row r="24" spans="1:5">
       <c r="A24" s="1" t="s">
         <v>47</v>
       </c>
@@ -3703,7 +3702,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:5" hidden="1">
+    <row r="25" spans="1:5">
       <c r="A25" s="1" t="s">
         <v>51</v>
       </c>
@@ -3720,7 +3719,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" hidden="1">
+    <row r="26" spans="1:5">
       <c r="A26" s="1" t="s">
         <v>53</v>
       </c>
@@ -3737,7 +3736,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" hidden="1">
+    <row r="27" spans="1:5">
       <c r="A27" s="1" t="s">
         <v>55</v>
       </c>
@@ -3754,7 +3753,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:5" hidden="1">
+    <row r="28" spans="1:5">
       <c r="A28" s="1" t="s">
         <v>57</v>
       </c>
@@ -3771,7 +3770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:5" hidden="1">
+    <row r="29" spans="1:5">
       <c r="A29" s="1" t="s">
         <v>59</v>
       </c>
@@ -3805,7 +3804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1">
+    <row r="31" spans="1:5">
       <c r="A31" s="1" t="s">
         <v>63</v>
       </c>
@@ -3822,7 +3821,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:5" hidden="1">
+    <row r="32" spans="1:5">
       <c r="A32" s="1" t="s">
         <v>65</v>
       </c>
@@ -3839,7 +3838,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="33" spans="1:5" hidden="1">
+    <row r="33" spans="1:5">
       <c r="A33" s="1" t="s">
         <v>67</v>
       </c>
@@ -3873,7 +3872,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="35" spans="1:5" hidden="1">
+    <row r="35" spans="1:5">
       <c r="A35" s="1" t="s">
         <v>71</v>
       </c>
@@ -3890,7 +3889,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:5" hidden="1">
+    <row r="36" spans="1:5">
       <c r="A36" s="1" t="s">
         <v>73</v>
       </c>
@@ -3907,7 +3906,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" hidden="1">
+    <row r="37" spans="1:5">
       <c r="A37" s="1" t="s">
         <v>75</v>
       </c>
@@ -3924,7 +3923,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" hidden="1">
+    <row r="38" spans="1:5">
       <c r="A38" s="1" t="s">
         <v>77</v>
       </c>
@@ -3941,7 +3940,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="39" spans="1:5" hidden="1">
+    <row r="39" spans="1:5">
       <c r="A39" s="1" t="s">
         <v>79</v>
       </c>
@@ -3958,7 +3957,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" hidden="1">
+    <row r="40" spans="1:5">
       <c r="A40" s="1" t="s">
         <v>82</v>
       </c>
@@ -3992,7 +3991,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="42" spans="1:5" hidden="1">
+    <row r="42" spans="1:5">
       <c r="A42" s="1" t="s">
         <v>86</v>
       </c>
@@ -4009,7 +4008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:5" hidden="1">
+    <row r="43" spans="1:5">
       <c r="A43" s="1" t="s">
         <v>88</v>
       </c>
@@ -4020,7 +4019,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="44" spans="1:5" hidden="1">
+    <row r="44" spans="1:5">
       <c r="A44" s="1" t="s">
         <v>90</v>
       </c>
@@ -4037,7 +4036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:5" hidden="1">
+    <row r="45" spans="1:5">
       <c r="A45" s="1" t="s">
         <v>92</v>
       </c>
@@ -4054,7 +4053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:5" hidden="1">
+    <row r="46" spans="1:5">
       <c r="A46" s="1" t="s">
         <v>94</v>
       </c>
@@ -4071,7 +4070,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:5" hidden="1">
+    <row r="47" spans="1:5">
       <c r="A47" s="1" t="s">
         <v>96</v>
       </c>
@@ -4088,7 +4087,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:5" hidden="1">
+    <row r="48" spans="1:5">
       <c r="A48" s="1" t="s">
         <v>98</v>
       </c>
@@ -4105,7 +4104,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" hidden="1">
+    <row r="49" spans="1:5">
       <c r="A49" s="1" t="s">
         <v>100</v>
       </c>
@@ -4122,7 +4121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:5" hidden="1">
+    <row r="50" spans="1:5">
       <c r="A50" s="1" t="s">
         <v>102</v>
       </c>
@@ -4139,7 +4138,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:5" hidden="1">
+    <row r="51" spans="1:5">
       <c r="A51" s="1" t="s">
         <v>104</v>
       </c>
@@ -4156,7 +4155,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="52" spans="1:5" hidden="1">
+    <row r="52" spans="1:5">
       <c r="A52" s="1" t="s">
         <v>106</v>
       </c>
@@ -4173,7 +4172,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" hidden="1">
+    <row r="53" spans="1:5">
       <c r="A53" s="1" t="s">
         <v>108</v>
       </c>
@@ -4190,7 +4189,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:5" hidden="1">
+    <row r="54" spans="1:5">
       <c r="A54" s="1" t="s">
         <v>110</v>
       </c>
@@ -4207,7 +4206,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="55" spans="1:5" hidden="1">
+    <row r="55" spans="1:5">
       <c r="A55" s="1" t="s">
         <v>112</v>
       </c>
@@ -4224,7 +4223,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" hidden="1">
+    <row r="56" spans="1:5">
       <c r="A56" s="1" t="s">
         <v>114</v>
       </c>
@@ -4241,7 +4240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:5" hidden="1">
+    <row r="57" spans="1:5">
       <c r="A57" s="1" t="s">
         <v>116</v>
       </c>
@@ -4258,7 +4257,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="58" spans="1:5" hidden="1">
+    <row r="58" spans="1:5">
       <c r="A58" s="1" t="s">
         <v>118</v>
       </c>
@@ -4275,7 +4274,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:5" hidden="1">
+    <row r="59" spans="1:5">
       <c r="A59" s="1" t="s">
         <v>120</v>
       </c>
@@ -4292,7 +4291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:5" hidden="1">
+    <row r="60" spans="1:5">
       <c r="A60" s="1" t="s">
         <v>122</v>
       </c>
@@ -4309,7 +4308,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:5" hidden="1">
+    <row r="61" spans="1:5">
       <c r="A61" s="1" t="s">
         <v>124</v>
       </c>
@@ -4326,7 +4325,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:5" hidden="1">
+    <row r="62" spans="1:5">
       <c r="A62" s="1" t="s">
         <v>126</v>
       </c>
@@ -4343,7 +4342,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:5" hidden="1">
+    <row r="63" spans="1:5">
       <c r="A63" s="1" t="s">
         <v>128</v>
       </c>
@@ -4360,7 +4359,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="64" spans="1:5" hidden="1">
+    <row r="64" spans="1:5">
       <c r="A64" s="1" t="s">
         <v>130</v>
       </c>
@@ -4377,7 +4376,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:5" hidden="1">
+    <row r="65" spans="1:5">
       <c r="A65" s="1" t="s">
         <v>132</v>
       </c>
@@ -4394,7 +4393,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="66" spans="1:5" hidden="1">
+    <row r="66" spans="1:5">
       <c r="A66" s="1" t="s">
         <v>134</v>
       </c>
@@ -4411,7 +4410,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" hidden="1">
+    <row r="67" spans="1:5">
       <c r="A67" s="1" t="s">
         <v>136</v>
       </c>
@@ -4428,7 +4427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:5" hidden="1">
+    <row r="68" spans="1:5">
       <c r="A68" s="1" t="s">
         <v>138</v>
       </c>
@@ -4445,7 +4444,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:5" hidden="1">
+    <row r="69" spans="1:5">
       <c r="A69" s="1" t="s">
         <v>140</v>
       </c>
@@ -4462,7 +4461,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:5" hidden="1">
+    <row r="70" spans="1:5">
       <c r="A70" s="1" t="s">
         <v>142</v>
       </c>
@@ -4479,7 +4478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:5" hidden="1">
+    <row r="71" spans="1:5">
       <c r="A71" s="1" t="s">
         <v>145</v>
       </c>
@@ -4496,7 +4495,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:5" hidden="1">
+    <row r="72" spans="1:5">
       <c r="A72" s="1" t="s">
         <v>147</v>
       </c>
@@ -4513,7 +4512,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="1:5" hidden="1">
+    <row r="73" spans="1:5">
       <c r="A73" s="1" t="s">
         <v>149</v>
       </c>
@@ -4530,7 +4529,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="1:5" hidden="1">
+    <row r="74" spans="1:5">
       <c r="A74" s="1" t="s">
         <v>151</v>
       </c>
@@ -4547,7 +4546,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="1:5" hidden="1">
+    <row r="75" spans="1:5">
       <c r="A75" s="1" t="s">
         <v>153</v>
       </c>
@@ -4564,7 +4563,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="76" spans="1:5" hidden="1">
+    <row r="76" spans="1:5">
       <c r="A76" s="1" t="s">
         <v>155</v>
       </c>
@@ -4581,7 +4580,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="77" spans="1:5" hidden="1">
+    <row r="77" spans="1:5">
       <c r="A77" s="1" t="s">
         <v>157</v>
       </c>
@@ -4598,7 +4597,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:5" hidden="1">
+    <row r="78" spans="1:5">
       <c r="A78" s="1" t="s">
         <v>159</v>
       </c>
@@ -4615,7 +4614,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="79" spans="1:5" hidden="1">
+    <row r="79" spans="1:5">
       <c r="A79" s="1" t="s">
         <v>163</v>
       </c>
@@ -4632,7 +4631,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="1:5" hidden="1">
+    <row r="80" spans="1:5">
       <c r="A80" s="1" t="s">
         <v>165</v>
       </c>
@@ -4649,7 +4648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:5" hidden="1">
+    <row r="81" spans="1:5">
       <c r="A81" s="1" t="s">
         <v>167</v>
       </c>
@@ -4683,7 +4682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:5" hidden="1">
+    <row r="83" spans="1:5">
       <c r="A83" s="1" t="s">
         <v>171</v>
       </c>
@@ -4700,7 +4699,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="84" spans="1:5" hidden="1">
+    <row r="84" spans="1:5">
       <c r="A84" s="1" t="s">
         <v>173</v>
       </c>
@@ -4717,7 +4716,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:5" hidden="1">
+    <row r="85" spans="1:5">
       <c r="A85" s="1" t="s">
         <v>175</v>
       </c>
@@ -4734,7 +4733,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="86" spans="1:5" hidden="1">
+    <row r="86" spans="1:5">
       <c r="A86" s="1" t="s">
         <v>177</v>
       </c>
@@ -4751,7 +4750,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="87" spans="1:5" hidden="1">
+    <row r="87" spans="1:5">
       <c r="A87" s="1" t="s">
         <v>179</v>
       </c>
@@ -4768,7 +4767,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="88" spans="1:5" hidden="1">
+    <row r="88" spans="1:5">
       <c r="A88" s="1" t="s">
         <v>181</v>
       </c>
@@ -4785,7 +4784,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="89" spans="1:5" hidden="1">
+    <row r="89" spans="1:5">
       <c r="A89" s="1" t="s">
         <v>183</v>
       </c>
@@ -4802,7 +4801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:5" hidden="1">
+    <row r="90" spans="1:5">
       <c r="A90" s="1" t="s">
         <v>185</v>
       </c>
@@ -4819,7 +4818,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="91" spans="1:5" hidden="1">
+    <row r="91" spans="1:5">
       <c r="A91" s="1" t="s">
         <v>187</v>
       </c>
@@ -4836,7 +4835,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="92" spans="1:5" hidden="1">
+    <row r="92" spans="1:5">
       <c r="A92" s="1" t="s">
         <v>189</v>
       </c>
@@ -4870,7 +4869,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="94" spans="1:5" hidden="1">
+    <row r="94" spans="1:5">
       <c r="A94" s="1" t="s">
         <v>193</v>
       </c>
@@ -4887,7 +4886,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="95" spans="1:5" hidden="1">
+    <row r="95" spans="1:5">
       <c r="A95" s="1" t="s">
         <v>195</v>
       </c>
@@ -4904,7 +4903,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:5" hidden="1">
+    <row r="96" spans="1:5">
       <c r="A96" s="1" t="s">
         <v>197</v>
       </c>
@@ -4921,7 +4920,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="97" spans="1:5" hidden="1">
+    <row r="97" spans="1:5">
       <c r="A97" s="1" t="s">
         <v>199</v>
       </c>
@@ -4938,7 +4937,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="98" spans="1:5" hidden="1">
+    <row r="98" spans="1:5">
       <c r="A98" s="1" t="s">
         <v>201</v>
       </c>
@@ -4955,7 +4954,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="99" spans="1:5" hidden="1">
+    <row r="99" spans="1:5">
       <c r="A99" s="1" t="s">
         <v>203</v>
       </c>
@@ -4972,7 +4971,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:5" hidden="1">
+    <row r="100" spans="1:5">
       <c r="A100" s="1" t="s">
         <v>205</v>
       </c>
@@ -4989,7 +4988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:5" hidden="1">
+    <row r="101" spans="1:5">
       <c r="A101" s="1" t="s">
         <v>207</v>
       </c>
@@ -5006,7 +5005,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:5" hidden="1">
+    <row r="102" spans="1:5">
       <c r="A102" s="1" t="s">
         <v>209</v>
       </c>
@@ -5023,7 +5022,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="103" spans="1:5" hidden="1">
+    <row r="103" spans="1:5">
       <c r="A103" s="1" t="s">
         <v>211</v>
       </c>
@@ -5040,7 +5039,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="104" spans="1:5" hidden="1">
+    <row r="104" spans="1:5">
       <c r="A104" s="1" t="s">
         <v>213</v>
       </c>
@@ -5057,7 +5056,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="105" spans="1:5" hidden="1">
+    <row r="105" spans="1:5">
       <c r="A105" s="1" t="s">
         <v>215</v>
       </c>
@@ -5074,7 +5073,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="106" spans="1:5" hidden="1">
+    <row r="106" spans="1:5">
       <c r="A106" s="1" t="s">
         <v>217</v>
       </c>
@@ -5091,7 +5090,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="107" spans="1:5" hidden="1">
+    <row r="107" spans="1:5">
       <c r="A107" s="1" t="s">
         <v>219</v>
       </c>
@@ -5108,7 +5107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:5" hidden="1">
+    <row r="108" spans="1:5">
       <c r="A108" s="1" t="s">
         <v>221</v>
       </c>
@@ -5125,7 +5124,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="109" spans="1:5" hidden="1">
+    <row r="109" spans="1:5">
       <c r="A109" s="1" t="s">
         <v>223</v>
       </c>
@@ -5142,7 +5141,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="110" spans="1:5" hidden="1">
+    <row r="110" spans="1:5">
       <c r="A110" s="1" t="s">
         <v>225</v>
       </c>
@@ -5159,7 +5158,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:5" hidden="1">
+    <row r="111" spans="1:5">
       <c r="A111" s="1" t="s">
         <v>227</v>
       </c>
@@ -5176,7 +5175,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:5" hidden="1">
+    <row r="112" spans="1:5">
       <c r="A112" s="1" t="s">
         <v>229</v>
       </c>
@@ -5193,7 +5192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:5" hidden="1">
+    <row r="113" spans="1:5">
       <c r="A113" s="1" t="s">
         <v>231</v>
       </c>
@@ -5210,7 +5209,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="114" spans="1:5" hidden="1">
+    <row r="114" spans="1:5">
       <c r="A114" s="1" t="s">
         <v>233</v>
       </c>
@@ -5227,7 +5226,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="115" spans="1:5" hidden="1">
+    <row r="115" spans="1:5">
       <c r="A115" s="1" t="s">
         <v>235</v>
       </c>
@@ -5244,7 +5243,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:5" hidden="1">
+    <row r="116" spans="1:5">
       <c r="A116" s="1" t="s">
         <v>237</v>
       </c>
@@ -5261,7 +5260,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="117" spans="1:5" hidden="1">
+    <row r="117" spans="1:5">
       <c r="A117" s="1" t="s">
         <v>239</v>
       </c>
@@ -5278,7 +5277,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="118" spans="1:5" hidden="1">
+    <row r="118" spans="1:5">
       <c r="A118" s="1" t="s">
         <v>241</v>
       </c>
@@ -5295,7 +5294,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:5" hidden="1">
+    <row r="119" spans="1:5">
       <c r="A119" s="1" t="s">
         <v>243</v>
       </c>
@@ -5312,7 +5311,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:5" hidden="1">
+    <row r="120" spans="1:5">
       <c r="A120" s="1" t="s">
         <v>245</v>
       </c>
@@ -5329,7 +5328,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:5" hidden="1">
+    <row r="121" spans="1:5">
       <c r="A121" s="1" t="s">
         <v>247</v>
       </c>
@@ -5346,7 +5345,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:5" hidden="1">
+    <row r="122" spans="1:5">
       <c r="A122" s="1" t="s">
         <v>249</v>
       </c>
@@ -5363,7 +5362,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:5" hidden="1">
+    <row r="123" spans="1:5">
       <c r="A123" s="1" t="s">
         <v>251</v>
       </c>
@@ -5380,7 +5379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:5" hidden="1">
+    <row r="124" spans="1:5">
       <c r="A124" s="1" t="s">
         <v>253</v>
       </c>
@@ -5397,7 +5396,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="125" spans="1:5" hidden="1">
+    <row r="125" spans="1:5">
       <c r="A125" s="1" t="s">
         <v>255</v>
       </c>
@@ -5414,7 +5413,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="126" spans="1:5" hidden="1">
+    <row r="126" spans="1:5">
       <c r="A126" s="1" t="s">
         <v>257</v>
       </c>
@@ -5431,7 +5430,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:5" hidden="1">
+    <row r="127" spans="1:5">
       <c r="A127" s="1" t="s">
         <v>259</v>
       </c>
@@ -5448,7 +5447,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="128" spans="1:5" hidden="1">
+    <row r="128" spans="1:5">
       <c r="A128" s="1" t="s">
         <v>261</v>
       </c>
@@ -5465,7 +5464,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="129" spans="1:5" hidden="1">
+    <row r="129" spans="1:5">
       <c r="A129" s="1" t="s">
         <v>263</v>
       </c>
@@ -5482,7 +5481,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="130" spans="1:5" hidden="1">
+    <row r="130" spans="1:5">
       <c r="A130" s="1" t="s">
         <v>265</v>
       </c>
@@ -5499,7 +5498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:5" hidden="1">
+    <row r="131" spans="1:5">
       <c r="A131" s="1" t="s">
         <v>267</v>
       </c>
@@ -5516,7 +5515,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="132" spans="1:5" hidden="1">
+    <row r="132" spans="1:5">
       <c r="A132" s="1" t="s">
         <v>270</v>
       </c>
@@ -5533,7 +5532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:5" hidden="1">
+    <row r="133" spans="1:5">
       <c r="A133" s="1" t="s">
         <v>272</v>
       </c>
@@ -5550,7 +5549,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="134" spans="1:5" hidden="1">
+    <row r="134" spans="1:5">
       <c r="A134" s="1" t="s">
         <v>274</v>
       </c>
@@ -5567,7 +5566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:5" hidden="1">
+    <row r="135" spans="1:5">
       <c r="A135" s="1" t="s">
         <v>276</v>
       </c>
@@ -5584,7 +5583,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:5" hidden="1">
+    <row r="136" spans="1:5">
       <c r="A136" s="1" t="s">
         <v>278</v>
       </c>
@@ -5601,7 +5600,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="137" spans="1:5" hidden="1">
+    <row r="137" spans="1:5">
       <c r="A137" s="1" t="s">
         <v>280</v>
       </c>
@@ -5618,7 +5617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:5" hidden="1">
+    <row r="138" spans="1:5">
       <c r="A138" s="1" t="s">
         <v>621</v>
       </c>
@@ -5669,7 +5668,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="141" spans="1:5" hidden="1">
+    <row r="141" spans="1:5">
       <c r="A141" s="1" t="s">
         <v>627</v>
       </c>
@@ -5677,7 +5676,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="142" spans="1:5" hidden="1">
+    <row r="142" spans="1:5">
       <c r="A142" s="1" t="s">
         <v>629</v>
       </c>
@@ -5694,7 +5693,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="143" spans="1:5" hidden="1">
+    <row r="143" spans="1:5">
       <c r="A143" s="1" t="s">
         <v>631</v>
       </c>
@@ -5711,7 +5710,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="144" spans="1:5" hidden="1">
+    <row r="144" spans="1:5">
       <c r="A144" s="1" t="s">
         <v>633</v>
       </c>
@@ -5722,7 +5721,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="145" spans="1:5" hidden="1">
+    <row r="145" spans="1:5">
       <c r="A145" s="1" t="s">
         <v>636</v>
       </c>
@@ -5739,7 +5738,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="146" spans="1:5" hidden="1">
+    <row r="146" spans="1:5">
       <c r="A146" s="1" t="s">
         <v>282</v>
       </c>
@@ -5756,7 +5755,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="147" spans="1:5" hidden="1">
+    <row r="147" spans="1:5">
       <c r="A147" s="1" t="s">
         <v>285</v>
       </c>
@@ -5773,7 +5772,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:5" hidden="1">
+    <row r="148" spans="1:5">
       <c r="A148" s="1" t="s">
         <v>287</v>
       </c>
@@ -5790,7 +5789,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="149" spans="1:5" hidden="1">
+    <row r="149" spans="1:5">
       <c r="A149" s="1" t="s">
         <v>289</v>
       </c>
@@ -5807,7 +5806,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="150" spans="1:5" hidden="1">
+    <row r="150" spans="1:5">
       <c r="A150" s="1" t="s">
         <v>291</v>
       </c>
@@ -5824,7 +5823,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="151" spans="1:5" hidden="1">
+    <row r="151" spans="1:5">
       <c r="A151" s="1" t="s">
         <v>293</v>
       </c>
@@ -5841,7 +5840,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="152" spans="1:5" hidden="1">
+    <row r="152" spans="1:5">
       <c r="A152" s="1" t="s">
         <v>295</v>
       </c>
@@ -5875,7 +5874,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="154" spans="1:5" hidden="1">
+    <row r="154" spans="1:5">
       <c r="A154" s="1" t="s">
         <v>299</v>
       </c>
@@ -5892,7 +5891,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="155" spans="1:5" hidden="1">
+    <row r="155" spans="1:5">
       <c r="A155" s="1" t="s">
         <v>303</v>
       </c>
@@ -5909,7 +5908,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:5" hidden="1">
+    <row r="156" spans="1:5">
       <c r="A156" s="1" t="s">
         <v>305</v>
       </c>
@@ -5926,7 +5925,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:5" hidden="1">
+    <row r="157" spans="1:5">
       <c r="A157" s="1" t="s">
         <v>307</v>
       </c>
@@ -5943,7 +5942,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="158" spans="1:5" hidden="1">
+    <row r="158" spans="1:5">
       <c r="A158" s="1" t="s">
         <v>310</v>
       </c>
@@ -5960,7 +5959,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="159" spans="1:5" hidden="1">
+    <row r="159" spans="1:5">
       <c r="A159" s="1" t="s">
         <v>312</v>
       </c>
@@ -5977,7 +5976,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="160" spans="1:5" hidden="1">
+    <row r="160" spans="1:5">
       <c r="A160" s="1" t="s">
         <v>314</v>
       </c>
@@ -5994,7 +5993,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="161" spans="1:5" hidden="1">
+    <row r="161" spans="1:5">
       <c r="A161" s="1" t="s">
         <v>316</v>
       </c>
@@ -6011,7 +6010,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:5" hidden="1">
+    <row r="162" spans="1:5">
       <c r="A162" s="1" t="s">
         <v>318</v>
       </c>
@@ -6028,7 +6027,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="163" spans="1:5" hidden="1">
+    <row r="163" spans="1:5">
       <c r="A163" s="1" t="s">
         <v>320</v>
       </c>
@@ -6045,7 +6044,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:5" hidden="1">
+    <row r="164" spans="1:5">
       <c r="A164" s="1" t="s">
         <v>322</v>
       </c>
@@ -6062,7 +6061,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:5" hidden="1">
+    <row r="165" spans="1:5">
       <c r="A165" s="1" t="s">
         <v>324</v>
       </c>
@@ -6079,7 +6078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:5" hidden="1">
+    <row r="166" spans="1:5">
       <c r="A166" s="1" t="s">
         <v>326</v>
       </c>
@@ -6096,7 +6095,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:5" hidden="1">
+    <row r="167" spans="1:5">
       <c r="A167" s="1" t="s">
         <v>328</v>
       </c>
@@ -6113,7 +6112,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="168" spans="1:5" hidden="1">
+    <row r="168" spans="1:5">
       <c r="A168" s="1" t="s">
         <v>330</v>
       </c>
@@ -6130,7 +6129,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:5" hidden="1">
+    <row r="169" spans="1:5">
       <c r="A169" s="1" t="s">
         <v>332</v>
       </c>
@@ -6147,7 +6146,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="170" spans="1:5" hidden="1">
+    <row r="170" spans="1:5">
       <c r="A170" s="1" t="s">
         <v>334</v>
       </c>
@@ -6164,7 +6163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:5" hidden="1">
+    <row r="171" spans="1:5">
       <c r="A171" s="1" t="s">
         <v>336</v>
       </c>
@@ -6181,7 +6180,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="172" spans="1:5" hidden="1">
+    <row r="172" spans="1:5">
       <c r="A172" s="1" t="s">
         <v>338</v>
       </c>
@@ -6198,7 +6197,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:5" hidden="1">
+    <row r="173" spans="1:5">
       <c r="A173" s="1" t="s">
         <v>340</v>
       </c>
@@ -6215,7 +6214,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:5" hidden="1">
+    <row r="174" spans="1:5">
       <c r="A174" s="1" t="s">
         <v>342</v>
       </c>
@@ -6232,7 +6231,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="175" spans="1:5" hidden="1">
+    <row r="175" spans="1:5">
       <c r="A175" s="1" t="s">
         <v>344</v>
       </c>
@@ -6249,7 +6248,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="176" spans="1:5" hidden="1">
+    <row r="176" spans="1:5">
       <c r="A176" s="1" t="s">
         <v>346</v>
       </c>
@@ -6266,7 +6265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="1:5" hidden="1">
+    <row r="177" spans="1:5">
       <c r="A177" s="1" t="s">
         <v>348</v>
       </c>
@@ -6283,7 +6282,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="178" spans="1:5" hidden="1">
+    <row r="178" spans="1:5">
       <c r="A178" s="1" t="s">
         <v>350</v>
       </c>
@@ -6300,7 +6299,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="179" spans="1:5" hidden="1">
+    <row r="179" spans="1:5">
       <c r="A179" s="1" t="s">
         <v>352</v>
       </c>
@@ -6317,7 +6316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="180" spans="1:5" hidden="1">
+    <row r="180" spans="1:5">
       <c r="A180" s="1" t="s">
         <v>354</v>
       </c>
@@ -6334,7 +6333,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="181" spans="1:5" hidden="1">
+    <row r="181" spans="1:5">
       <c r="A181" s="1" t="s">
         <v>356</v>
       </c>
@@ -6351,7 +6350,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="182" spans="1:5" hidden="1">
+    <row r="182" spans="1:5">
       <c r="A182" s="1" t="s">
         <v>358</v>
       </c>
@@ -6368,7 +6367,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="183" spans="1:5" hidden="1">
+    <row r="183" spans="1:5">
       <c r="A183" s="1" t="s">
         <v>360</v>
       </c>
@@ -6385,7 +6384,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="184" spans="1:5" hidden="1">
+    <row r="184" spans="1:5">
       <c r="A184" s="1" t="s">
         <v>362</v>
       </c>
@@ -6402,7 +6401,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="185" spans="1:5" hidden="1">
+    <row r="185" spans="1:5">
       <c r="A185" s="1" t="s">
         <v>364</v>
       </c>
@@ -6419,7 +6418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="186" spans="1:5" hidden="1">
+    <row r="186" spans="1:5">
       <c r="A186" s="1" t="s">
         <v>366</v>
       </c>
@@ -6436,7 +6435,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="187" spans="1:5" hidden="1">
+    <row r="187" spans="1:5">
       <c r="A187" s="1" t="s">
         <v>368</v>
       </c>
@@ -6453,7 +6452,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:5" hidden="1">
+    <row r="188" spans="1:5">
       <c r="A188" s="1" t="s">
         <v>370</v>
       </c>
@@ -6470,7 +6469,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:5" hidden="1">
+    <row r="189" spans="1:5">
       <c r="A189" s="1" t="s">
         <v>372</v>
       </c>
@@ -6487,7 +6486,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="190" spans="1:5" hidden="1">
+    <row r="190" spans="1:5">
       <c r="A190" s="1" t="s">
         <v>374</v>
       </c>
@@ -6504,7 +6503,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="191" spans="1:5" hidden="1">
+    <row r="191" spans="1:5">
       <c r="A191" s="1" t="s">
         <v>376</v>
       </c>
@@ -6521,7 +6520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:5" hidden="1">
+    <row r="192" spans="1:5">
       <c r="A192" s="1" t="s">
         <v>378</v>
       </c>
@@ -6538,7 +6537,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="193" spans="1:5" hidden="1">
+    <row r="193" spans="1:5">
       <c r="A193" s="1" t="s">
         <v>380</v>
       </c>
@@ -6555,7 +6554,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:5" hidden="1">
+    <row r="194" spans="1:5">
       <c r="A194" s="1" t="s">
         <v>382</v>
       </c>
@@ -6572,7 +6571,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="195" spans="1:5" hidden="1">
+    <row r="195" spans="1:5">
       <c r="A195" s="1" t="s">
         <v>384</v>
       </c>
@@ -6589,7 +6588,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="196" spans="1:5" hidden="1">
+    <row r="196" spans="1:5">
       <c r="A196" s="1" t="s">
         <v>386</v>
       </c>
@@ -6606,7 +6605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="197" spans="1:5" hidden="1">
+    <row r="197" spans="1:5">
       <c r="A197" s="1" t="s">
         <v>388</v>
       </c>
@@ -6623,7 +6622,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="198" spans="1:5" hidden="1">
+    <row r="198" spans="1:5">
       <c r="A198" s="1" t="s">
         <v>390</v>
       </c>
@@ -6640,7 +6639,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="199" spans="1:5" hidden="1">
+    <row r="199" spans="1:5">
       <c r="A199" s="1" t="s">
         <v>392</v>
       </c>
@@ -6657,7 +6656,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="200" spans="1:5" hidden="1">
+    <row r="200" spans="1:5">
       <c r="A200" s="1" t="s">
         <v>394</v>
       </c>
@@ -6674,7 +6673,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="201" spans="1:5" hidden="1">
+    <row r="201" spans="1:5">
       <c r="A201" s="1" t="s">
         <v>396</v>
       </c>
@@ -6691,7 +6690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="202" spans="1:5" hidden="1">
+    <row r="202" spans="1:5">
       <c r="A202" s="1" t="s">
         <v>398</v>
       </c>
@@ -6708,7 +6707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="203" spans="1:5" hidden="1">
+    <row r="203" spans="1:5">
       <c r="A203" s="1" t="s">
         <v>400</v>
       </c>
@@ -6725,7 +6724,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="204" spans="1:5" hidden="1">
+    <row r="204" spans="1:5">
       <c r="A204" s="1" t="s">
         <v>402</v>
       </c>
@@ -6742,7 +6741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:5" hidden="1">
+    <row r="205" spans="1:5">
       <c r="A205" s="1" t="s">
         <v>404</v>
       </c>
@@ -6759,7 +6758,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="206" spans="1:5" hidden="1">
+    <row r="206" spans="1:5">
       <c r="A206" s="1" t="s">
         <v>406</v>
       </c>
@@ -6776,7 +6775,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="1:5" hidden="1">
+    <row r="207" spans="1:5">
       <c r="A207" s="1" t="s">
         <v>408</v>
       </c>
@@ -6793,7 +6792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:5" hidden="1">
+    <row r="208" spans="1:5">
       <c r="A208" s="1" t="s">
         <v>410</v>
       </c>
@@ -6810,7 +6809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="1:5" hidden="1">
+    <row r="209" spans="1:5">
       <c r="A209" s="1" t="s">
         <v>412</v>
       </c>
@@ -6827,7 +6826,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="210" spans="1:5" hidden="1">
+    <row r="210" spans="1:5">
       <c r="A210" s="1" t="s">
         <v>414</v>
       </c>
@@ -6844,7 +6843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="1:5" hidden="1">
+    <row r="211" spans="1:5">
       <c r="A211" s="1" t="s">
         <v>416</v>
       </c>
@@ -6861,7 +6860,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="212" spans="1:5" hidden="1">
+    <row r="212" spans="1:5">
       <c r="A212" s="1" t="s">
         <v>418</v>
       </c>
@@ -6878,7 +6877,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="213" spans="1:5" hidden="1">
+    <row r="213" spans="1:5">
       <c r="A213" s="1" t="s">
         <v>420</v>
       </c>
@@ -6895,7 +6894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="214" spans="1:5" hidden="1">
+    <row r="214" spans="1:5">
       <c r="A214" s="1" t="s">
         <v>422</v>
       </c>
@@ -6912,7 +6911,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="215" spans="1:5" hidden="1">
+    <row r="215" spans="1:5">
       <c r="A215" s="1" t="s">
         <v>424</v>
       </c>
@@ -6929,7 +6928,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="216" spans="1:5" hidden="1">
+    <row r="216" spans="1:5">
       <c r="A216" s="1" t="s">
         <v>426</v>
       </c>
@@ -6946,7 +6945,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="217" spans="1:5" hidden="1">
+    <row r="217" spans="1:5">
       <c r="A217" s="1" t="s">
         <v>428</v>
       </c>
@@ -6963,7 +6962,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="218" spans="1:5" hidden="1">
+    <row r="218" spans="1:5">
       <c r="A218" s="1" t="s">
         <v>430</v>
       </c>
@@ -6980,7 +6979,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="219" spans="1:5" hidden="1">
+    <row r="219" spans="1:5">
       <c r="A219" s="1" t="s">
         <v>432</v>
       </c>
@@ -6997,7 +6996,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="220" spans="1:5" hidden="1">
+    <row r="220" spans="1:5">
       <c r="A220" s="1" t="s">
         <v>434</v>
       </c>
@@ -7014,7 +7013,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="221" spans="1:5" hidden="1">
+    <row r="221" spans="1:5">
       <c r="A221" s="1" t="s">
         <v>436</v>
       </c>
@@ -7031,7 +7030,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="222" spans="1:5" hidden="1">
+    <row r="222" spans="1:5">
       <c r="A222" s="1" t="s">
         <v>438</v>
       </c>
@@ -7048,7 +7047,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="223" spans="1:5" hidden="1">
+    <row r="223" spans="1:5">
       <c r="A223" s="1" t="s">
         <v>440</v>
       </c>
@@ -7065,7 +7064,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="224" spans="1:5" hidden="1">
+    <row r="224" spans="1:5">
       <c r="A224" s="1" t="s">
         <v>442</v>
       </c>
@@ -7082,7 +7081,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="225" spans="1:5" hidden="1">
+    <row r="225" spans="1:5">
       <c r="A225" s="1" t="s">
         <v>444</v>
       </c>
@@ -7099,7 +7098,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="226" spans="1:5" hidden="1">
+    <row r="226" spans="1:5">
       <c r="A226" s="1" t="s">
         <v>446</v>
       </c>
@@ -7116,7 +7115,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="227" spans="1:5" hidden="1">
+    <row r="227" spans="1:5">
       <c r="A227" s="1" t="s">
         <v>448</v>
       </c>
@@ -7133,7 +7132,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="228" spans="1:5" hidden="1">
+    <row r="228" spans="1:5">
       <c r="A228" s="1" t="s">
         <v>450</v>
       </c>
@@ -7150,7 +7149,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:5" hidden="1">
+    <row r="229" spans="1:5">
       <c r="A229" s="1" t="s">
         <v>452</v>
       </c>
@@ -7167,7 +7166,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="230" spans="1:5" hidden="1">
+    <row r="230" spans="1:5">
       <c r="A230" s="1" t="s">
         <v>454</v>
       </c>
@@ -7184,7 +7183,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231" spans="1:5" hidden="1">
+    <row r="231" spans="1:5">
       <c r="A231" s="1" t="s">
         <v>456</v>
       </c>
@@ -7201,7 +7200,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="232" spans="1:5" hidden="1">
+    <row r="232" spans="1:5">
       <c r="A232" s="1" t="s">
         <v>458</v>
       </c>
@@ -7218,7 +7217,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="233" spans="1:5" hidden="1">
+    <row r="233" spans="1:5">
       <c r="A233" s="1" t="s">
         <v>460</v>
       </c>
@@ -7235,7 +7234,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="234" spans="1:5" hidden="1">
+    <row r="234" spans="1:5">
       <c r="A234" s="1" t="s">
         <v>462</v>
       </c>
@@ -7252,7 +7251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="1:5" hidden="1">
+    <row r="235" spans="1:5">
       <c r="A235" s="1" t="s">
         <v>464</v>
       </c>
@@ -7269,7 +7268,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="236" spans="1:5" hidden="1">
+    <row r="236" spans="1:5">
       <c r="A236" s="1" t="s">
         <v>466</v>
       </c>
@@ -7286,7 +7285,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="237" spans="1:5" hidden="1">
+    <row r="237" spans="1:5">
       <c r="A237" s="1" t="s">
         <v>468</v>
       </c>
@@ -7303,7 +7302,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="238" spans="1:5" hidden="1">
+    <row r="238" spans="1:5">
       <c r="A238" s="1" t="s">
         <v>470</v>
       </c>
@@ -7320,7 +7319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="239" spans="1:5" hidden="1">
+    <row r="239" spans="1:5">
       <c r="A239" s="1" t="s">
         <v>472</v>
       </c>
@@ -7337,7 +7336,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="240" spans="1:5" hidden="1">
+    <row r="240" spans="1:5">
       <c r="A240" s="1" t="s">
         <v>474</v>
       </c>
@@ -7354,7 +7353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="241" spans="1:5" hidden="1">
+    <row r="241" spans="1:5">
       <c r="A241" s="1" t="s">
         <v>476</v>
       </c>
@@ -7371,7 +7370,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="242" spans="1:5" hidden="1">
+    <row r="242" spans="1:5">
       <c r="A242" s="1" t="s">
         <v>478</v>
       </c>
@@ -7388,7 +7387,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="243" spans="1:5" hidden="1">
+    <row r="243" spans="1:5">
       <c r="A243" s="1" t="s">
         <v>480</v>
       </c>
@@ -7405,7 +7404,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="244" spans="1:5" hidden="1">
+    <row r="244" spans="1:5">
       <c r="A244" s="1" t="s">
         <v>482</v>
       </c>
@@ -7422,7 +7421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="245" spans="1:5" hidden="1">
+    <row r="245" spans="1:5">
       <c r="A245" s="1" t="s">
         <v>484</v>
       </c>
@@ -7456,7 +7455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="1:5" hidden="1">
+    <row r="247" spans="1:5">
       <c r="A247" s="1" t="s">
         <v>488</v>
       </c>
@@ -7473,7 +7472,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="248" spans="1:5" hidden="1">
+    <row r="248" spans="1:5">
       <c r="A248" s="1" t="s">
         <v>490</v>
       </c>
@@ -7490,7 +7489,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="249" spans="1:5" hidden="1">
+    <row r="249" spans="1:5">
       <c r="A249" s="1" t="s">
         <v>492</v>
       </c>
@@ -7507,7 +7506,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="250" spans="1:5" hidden="1">
+    <row r="250" spans="1:5">
       <c r="A250" s="1" t="s">
         <v>493</v>
       </c>
@@ -7524,7 +7523,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="251" spans="1:5" hidden="1">
+    <row r="251" spans="1:5">
       <c r="A251" s="1" t="s">
         <v>494</v>
       </c>
@@ -7541,7 +7540,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="252" spans="1:5" hidden="1">
+    <row r="252" spans="1:5">
       <c r="A252" s="1" t="s">
         <v>496</v>
       </c>
@@ -7558,7 +7557,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="253" spans="1:5" hidden="1">
+    <row r="253" spans="1:5">
       <c r="A253" s="1" t="s">
         <v>498</v>
       </c>
@@ -7575,7 +7574,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="254" spans="1:5" hidden="1">
+    <row r="254" spans="1:5">
       <c r="A254" s="1" t="s">
         <v>500</v>
       </c>
@@ -7592,7 +7591,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="255" spans="1:5" hidden="1">
+    <row r="255" spans="1:5">
       <c r="A255" s="1" t="s">
         <v>502</v>
       </c>
@@ -7609,7 +7608,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="256" spans="1:5" hidden="1">
+    <row r="256" spans="1:5">
       <c r="A256" s="1" t="s">
         <v>504</v>
       </c>
@@ -7626,7 +7625,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="257" spans="1:5" hidden="1">
+    <row r="257" spans="1:5">
       <c r="A257" s="1" t="s">
         <v>506</v>
       </c>
@@ -7643,7 +7642,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="258" spans="1:5" hidden="1">
+    <row r="258" spans="1:5">
       <c r="A258" s="1" t="s">
         <v>508</v>
       </c>
@@ -7660,7 +7659,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="259" spans="1:5" hidden="1">
+    <row r="259" spans="1:5">
       <c r="A259" s="1" t="s">
         <v>510</v>
       </c>
@@ -7677,7 +7676,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="260" spans="1:5" hidden="1">
+    <row r="260" spans="1:5">
       <c r="A260" s="1" t="s">
         <v>512</v>
       </c>
@@ -7694,7 +7693,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="261" spans="1:5" hidden="1">
+    <row r="261" spans="1:5">
       <c r="A261" s="1" t="s">
         <v>514</v>
       </c>
@@ -7711,7 +7710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="262" spans="1:5" hidden="1">
+    <row r="262" spans="1:5">
       <c r="A262" s="1" t="s">
         <v>516</v>
       </c>
@@ -7728,7 +7727,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="263" spans="1:5" hidden="1">
+    <row r="263" spans="1:5">
       <c r="A263" s="1" t="s">
         <v>518</v>
       </c>
@@ -7745,7 +7744,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="264" spans="1:5" hidden="1">
+    <row r="264" spans="1:5">
       <c r="A264" s="1" t="s">
         <v>520</v>
       </c>
@@ -7762,7 +7761,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="265" spans="1:5" hidden="1">
+    <row r="265" spans="1:5">
       <c r="A265" s="1" t="s">
         <v>522</v>
       </c>
@@ -7779,7 +7778,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="266" spans="1:5" hidden="1">
+    <row r="266" spans="1:5">
       <c r="A266" s="1" t="s">
         <v>524</v>
       </c>
@@ -7796,7 +7795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="267" spans="1:5" hidden="1">
+    <row r="267" spans="1:5">
       <c r="A267" s="1" t="s">
         <v>526</v>
       </c>
@@ -7813,7 +7812,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="268" spans="1:5" hidden="1">
+    <row r="268" spans="1:5">
       <c r="A268" s="1" t="s">
         <v>528</v>
       </c>
@@ -7830,7 +7829,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="269" spans="1:5" hidden="1">
+    <row r="269" spans="1:5">
       <c r="A269" s="1" t="s">
         <v>530</v>
       </c>
@@ -7847,7 +7846,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="270" spans="1:5" hidden="1">
+    <row r="270" spans="1:5">
       <c r="A270" s="1" t="s">
         <v>532</v>
       </c>
@@ -7864,7 +7863,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="271" spans="1:5" hidden="1">
+    <row r="271" spans="1:5">
       <c r="A271" s="1" t="s">
         <v>534</v>
       </c>
@@ -7881,7 +7880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="272" spans="1:5" hidden="1">
+    <row r="272" spans="1:5">
       <c r="A272" s="1" t="s">
         <v>536</v>
       </c>
@@ -7898,7 +7897,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="273" spans="1:5" hidden="1">
+    <row r="273" spans="1:5">
       <c r="A273" s="1" t="s">
         <v>538</v>
       </c>
@@ -7915,7 +7914,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="274" spans="1:5" hidden="1">
+    <row r="274" spans="1:5">
       <c r="A274" s="1" t="s">
         <v>540</v>
       </c>
@@ -7932,7 +7931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="275" spans="1:5" hidden="1">
+    <row r="275" spans="1:5">
       <c r="A275" s="1" t="s">
         <v>542</v>
       </c>
@@ -7949,7 +7948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="276" spans="1:5" hidden="1">
+    <row r="276" spans="1:5">
       <c r="A276" s="1" t="s">
         <v>544</v>
       </c>
@@ -7966,7 +7965,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="277" spans="1:5" hidden="1">
+    <row r="277" spans="1:5">
       <c r="A277" s="1" t="s">
         <v>546</v>
       </c>
@@ -7983,7 +7982,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="278" spans="1:5" hidden="1">
+    <row r="278" spans="1:5">
       <c r="A278" s="1" t="s">
         <v>548</v>
       </c>
@@ -8000,7 +7999,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="279" spans="1:5" hidden="1">
+    <row r="279" spans="1:5">
       <c r="A279" s="1" t="s">
         <v>550</v>
       </c>
@@ -8017,7 +8016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="280" spans="1:5" hidden="1">
+    <row r="280" spans="1:5">
       <c r="A280" s="1" t="s">
         <v>552</v>
       </c>
@@ -8034,7 +8033,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="281" spans="1:5" hidden="1">
+    <row r="281" spans="1:5">
       <c r="A281" s="1" t="s">
         <v>554</v>
       </c>
@@ -8051,7 +8050,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="282" spans="1:5" hidden="1">
+    <row r="282" spans="1:5">
       <c r="A282" s="1" t="s">
         <v>556</v>
       </c>
@@ -8068,7 +8067,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="283" spans="1:5" hidden="1">
+    <row r="283" spans="1:5">
       <c r="A283" s="1" t="s">
         <v>558</v>
       </c>
@@ -8085,7 +8084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="284" spans="1:5" hidden="1">
+    <row r="284" spans="1:5">
       <c r="A284" s="1" t="s">
         <v>560</v>
       </c>
@@ -8102,7 +8101,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="285" spans="1:5" hidden="1">
+    <row r="285" spans="1:5">
       <c r="A285" s="1" t="s">
         <v>562</v>
       </c>
@@ -8119,7 +8118,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="286" spans="1:5" hidden="1">
+    <row r="286" spans="1:5">
       <c r="A286" s="1" t="s">
         <v>564</v>
       </c>
@@ -8136,7 +8135,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="287" spans="1:5" hidden="1">
+    <row r="287" spans="1:5">
       <c r="A287" s="1" t="s">
         <v>566</v>
       </c>
@@ -8153,7 +8152,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="288" spans="1:5" hidden="1">
+    <row r="288" spans="1:5">
       <c r="A288" s="1" t="s">
         <v>568</v>
       </c>
@@ -8170,7 +8169,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="289" spans="1:5" hidden="1">
+    <row r="289" spans="1:5">
       <c r="A289" s="1" t="s">
         <v>570</v>
       </c>
@@ -8187,7 +8186,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="290" spans="1:5" hidden="1">
+    <row r="290" spans="1:5">
       <c r="A290" s="1" t="s">
         <v>572</v>
       </c>
@@ -8204,7 +8203,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="291" spans="1:5" hidden="1">
+    <row r="291" spans="1:5">
       <c r="A291" s="1" t="s">
         <v>574</v>
       </c>
@@ -8221,7 +8220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="292" spans="1:5" hidden="1">
+    <row r="292" spans="1:5">
       <c r="A292" s="1" t="s">
         <v>576</v>
       </c>
@@ -8238,7 +8237,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="293" spans="1:5" hidden="1">
+    <row r="293" spans="1:5">
       <c r="A293" s="1" t="s">
         <v>578</v>
       </c>
@@ -8255,7 +8254,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="294" spans="1:5" hidden="1">
+    <row r="294" spans="1:5">
       <c r="A294" s="1" t="s">
         <v>580</v>
       </c>
@@ -8272,7 +8271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="295" spans="1:5" hidden="1">
+    <row r="295" spans="1:5">
       <c r="A295" s="1" t="s">
         <v>582</v>
       </c>
@@ -8289,7 +8288,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="296" spans="1:5" hidden="1">
+    <row r="296" spans="1:5">
       <c r="A296" s="1" t="s">
         <v>584</v>
       </c>
@@ -8306,7 +8305,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="297" spans="1:5" hidden="1">
+    <row r="297" spans="1:5">
       <c r="A297" s="1" t="s">
         <v>586</v>
       </c>
@@ -8323,7 +8322,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="298" spans="1:5" hidden="1">
+    <row r="298" spans="1:5">
       <c r="A298" s="1" t="s">
         <v>588</v>
       </c>
@@ -8340,7 +8339,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="299" spans="1:5" hidden="1">
+    <row r="299" spans="1:5">
       <c r="A299" s="1" t="s">
         <v>592</v>
       </c>
@@ -8357,7 +8356,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="300" spans="1:5" hidden="1">
+    <row r="300" spans="1:5">
       <c r="A300" s="1" t="s">
         <v>600</v>
       </c>
@@ -8374,7 +8373,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="301" spans="1:5" hidden="1">
+    <row r="301" spans="1:5">
       <c r="A301" s="1" t="s">
         <v>590</v>
       </c>
@@ -8391,7 +8390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="302" spans="1:5" hidden="1">
+    <row r="302" spans="1:5">
       <c r="A302" s="1" t="s">
         <v>596</v>
       </c>
@@ -8408,7 +8407,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="303" spans="1:5" hidden="1">
+    <row r="303" spans="1:5">
       <c r="A303" s="1" t="s">
         <v>594</v>
       </c>
@@ -8425,7 +8424,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="304" spans="1:5" hidden="1">
+    <row r="304" spans="1:5">
       <c r="A304" s="1" t="s">
         <v>598</v>
       </c>
@@ -8442,7 +8441,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="305" spans="1:5" hidden="1">
+    <row r="305" spans="1:5">
       <c r="A305" s="1" t="s">
         <v>603</v>
       </c>
@@ -8459,7 +8458,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="306" spans="1:5" hidden="1">
+    <row r="306" spans="1:5">
       <c r="A306" s="1" t="s">
         <v>606</v>
       </c>
@@ -8476,7 +8475,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="307" spans="1:5" hidden="1">
+    <row r="307" spans="1:5">
       <c r="A307" s="1" t="s">
         <v>608</v>
       </c>
@@ -8493,7 +8492,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="308" spans="1:5" hidden="1">
+    <row r="308" spans="1:5">
       <c r="A308" s="1" t="s">
         <v>610</v>
       </c>
@@ -8510,7 +8509,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="309" spans="1:5" hidden="1">
+    <row r="309" spans="1:5">
       <c r="A309" s="1" t="s">
         <v>612</v>
       </c>
@@ -8527,7 +8526,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="310" spans="1:5" hidden="1">
+    <row r="310" spans="1:5">
       <c r="A310" s="1" t="s">
         <v>614</v>
       </c>
@@ -8544,7 +8543,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="311" spans="1:5" hidden="1">
+    <row r="311" spans="1:5">
       <c r="A311" s="1" t="s">
         <v>640</v>
       </c>
@@ -8561,7 +8560,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="312" spans="1:5" hidden="1">
+    <row r="312" spans="1:5">
       <c r="A312" s="1" t="s">
         <v>642</v>
       </c>
@@ -8578,7 +8577,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="313" spans="1:5" hidden="1">
+    <row r="313" spans="1:5">
       <c r="A313" s="1" t="s">
         <v>644</v>
       </c>
@@ -8595,7 +8594,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="314" spans="1:5" hidden="1">
+    <row r="314" spans="1:5">
       <c r="A314" s="1" t="s">
         <v>646</v>
       </c>
@@ -8612,7 +8611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="315" spans="1:5" hidden="1">
+    <row r="315" spans="1:5">
       <c r="A315" s="1" t="s">
         <v>648</v>
       </c>
@@ -8629,7 +8628,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="316" spans="1:5" hidden="1">
+    <row r="316" spans="1:5">
       <c r="A316" s="1" t="s">
         <v>650</v>
       </c>
@@ -8646,7 +8645,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="317" spans="1:5" hidden="1">
+    <row r="317" spans="1:5">
       <c r="A317" s="1" t="s">
         <v>652</v>
       </c>
@@ -8663,7 +8662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="318" spans="1:5" hidden="1">
+    <row r="318" spans="1:5">
       <c r="A318" s="1" t="s">
         <v>654</v>
       </c>
@@ -8680,7 +8679,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="319" spans="1:5" hidden="1">
+    <row r="319" spans="1:5">
       <c r="A319" s="1" t="s">
         <v>656</v>
       </c>
@@ -8697,7 +8696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="320" spans="1:5" hidden="1">
+    <row r="320" spans="1:5">
       <c r="A320" s="1" t="s">
         <v>658</v>
       </c>
@@ -8714,7 +8713,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="321" spans="1:5" hidden="1">
+    <row r="321" spans="1:5">
       <c r="A321" s="1" t="s">
         <v>660</v>
       </c>
@@ -8731,7 +8730,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="322" spans="1:5" hidden="1">
+    <row r="322" spans="1:5">
       <c r="A322" s="1" t="s">
         <v>662</v>
       </c>
@@ -8748,7 +8747,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="323" spans="1:5" hidden="1">
+    <row r="323" spans="1:5">
       <c r="A323" s="1" t="s">
         <v>664</v>
       </c>
@@ -8765,7 +8764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="324" spans="1:5" hidden="1">
+    <row r="324" spans="1:5">
       <c r="A324" s="1" t="s">
         <v>666</v>
       </c>
@@ -8782,7 +8781,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="325" spans="1:5" hidden="1">
+    <row r="325" spans="1:5">
       <c r="A325" s="1" t="s">
         <v>668</v>
       </c>
@@ -8799,7 +8798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="326" spans="1:5" hidden="1">
+    <row r="326" spans="1:5">
       <c r="A326" s="1" t="s">
         <v>670</v>
       </c>
@@ -8816,7 +8815,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="327" spans="1:5" hidden="1">
+    <row r="327" spans="1:5">
       <c r="A327" s="1" t="s">
         <v>672</v>
       </c>
@@ -8833,7 +8832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="328" spans="1:5" hidden="1">
+    <row r="328" spans="1:5">
       <c r="A328" s="1" t="s">
         <v>674</v>
       </c>
@@ -8850,7 +8849,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="329" spans="1:5" hidden="1">
+    <row r="329" spans="1:5">
       <c r="A329" s="1" t="s">
         <v>676</v>
       </c>
@@ -8867,7 +8866,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="330" spans="1:5" hidden="1">
+    <row r="330" spans="1:5">
       <c r="A330" s="1" t="s">
         <v>678</v>
       </c>
@@ -8884,7 +8883,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="331" spans="1:5" hidden="1">
+    <row r="331" spans="1:5">
       <c r="A331" s="1" t="s">
         <v>680</v>
       </c>
@@ -8901,7 +8900,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="332" spans="1:5" hidden="1">
+    <row r="332" spans="1:5">
       <c r="A332" s="1" t="s">
         <v>682</v>
       </c>
@@ -8918,7 +8917,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="333" spans="1:5" hidden="1">
+    <row r="333" spans="1:5">
       <c r="A333" s="1" t="s">
         <v>684</v>
       </c>
@@ -8935,7 +8934,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="334" spans="1:5" hidden="1">
+    <row r="334" spans="1:5">
       <c r="A334" s="1" t="s">
         <v>686</v>
       </c>
@@ -8952,7 +8951,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="335" spans="1:5" hidden="1">
+    <row r="335" spans="1:5">
       <c r="A335" s="1" t="s">
         <v>688</v>
       </c>
@@ -8969,7 +8968,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="336" spans="1:5" hidden="1">
+    <row r="336" spans="1:5">
       <c r="A336" s="1" t="s">
         <v>690</v>
       </c>
@@ -8986,7 +8985,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="337" spans="1:5" hidden="1">
+    <row r="337" spans="1:5">
       <c r="A337" s="1" t="s">
         <v>692</v>
       </c>
@@ -9003,7 +9002,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="338" spans="1:5" hidden="1">
+    <row r="338" spans="1:5">
       <c r="A338" s="1" t="s">
         <v>694</v>
       </c>
@@ -9020,7 +9019,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="339" spans="1:5" hidden="1">
+    <row r="339" spans="1:5">
       <c r="A339" s="1" t="s">
         <v>696</v>
       </c>
@@ -9037,7 +9036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="340" spans="1:5" hidden="1">
+    <row r="340" spans="1:5">
       <c r="A340" s="1" t="s">
         <v>698</v>
       </c>
@@ -9054,7 +9053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="341" spans="1:5" hidden="1">
+    <row r="341" spans="1:5">
       <c r="A341" s="1" t="s">
         <v>700</v>
       </c>
@@ -9071,7 +9070,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="342" spans="1:5" hidden="1">
+    <row r="342" spans="1:5">
       <c r="A342" s="1" t="s">
         <v>702</v>
       </c>
@@ -9088,7 +9087,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="343" spans="1:5" hidden="1">
+    <row r="343" spans="1:5">
       <c r="A343" s="1" t="s">
         <v>705</v>
       </c>
@@ -9105,7 +9104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="344" spans="1:5" hidden="1">
+    <row r="344" spans="1:5">
       <c r="A344" s="1" t="s">
         <v>707</v>
       </c>
@@ -9122,7 +9121,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="345" spans="1:5" hidden="1">
+    <row r="345" spans="1:5">
       <c r="A345" s="1" t="s">
         <v>710</v>
       </c>
@@ -9139,7 +9138,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="346" spans="1:5" hidden="1">
+    <row r="346" spans="1:5">
       <c r="A346" s="1" t="s">
         <v>712</v>
       </c>
@@ -9156,7 +9155,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="347" spans="1:5" hidden="1">
+    <row r="347" spans="1:5">
       <c r="A347" s="1" t="s">
         <v>714</v>
       </c>
@@ -9173,7 +9172,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="348" spans="1:5" hidden="1">
+    <row r="348" spans="1:5">
       <c r="A348" s="1" t="s">
         <v>716</v>
       </c>
@@ -9190,7 +9189,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="349" spans="1:5" hidden="1">
+    <row r="349" spans="1:5">
       <c r="A349" s="1" t="s">
         <v>718</v>
       </c>
@@ -9207,7 +9206,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="350" spans="1:5" hidden="1">
+    <row r="350" spans="1:5">
       <c r="A350" s="1" t="s">
         <v>720</v>
       </c>
@@ -9224,7 +9223,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="351" spans="1:5" hidden="1">
+    <row r="351" spans="1:5">
       <c r="A351" s="1" t="s">
         <v>722</v>
       </c>
@@ -9241,7 +9240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="352" spans="1:5" hidden="1">
+    <row r="352" spans="1:5">
       <c r="A352" s="1" t="s">
         <v>724</v>
       </c>
@@ -9258,7 +9257,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="353" spans="1:5" hidden="1">
+    <row r="353" spans="1:5">
       <c r="A353" s="1" t="s">
         <v>726</v>
       </c>
@@ -9275,7 +9274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="354" spans="1:5" hidden="1">
+    <row r="354" spans="1:5">
       <c r="A354" s="1" t="s">
         <v>728</v>
       </c>
@@ -9292,7 +9291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="355" spans="1:5" hidden="1">
+    <row r="355" spans="1:5">
       <c r="A355" s="1" t="s">
         <v>730</v>
       </c>
@@ -9309,7 +9308,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="356" spans="1:5" hidden="1">
+    <row r="356" spans="1:5">
       <c r="A356" s="1" t="s">
         <v>732</v>
       </c>
@@ -9326,7 +9325,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="357" spans="1:5" hidden="1">
+    <row r="357" spans="1:5">
       <c r="A357" s="1" t="s">
         <v>734</v>
       </c>
@@ -9343,7 +9342,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="358" spans="1:5" hidden="1">
+    <row r="358" spans="1:5">
       <c r="A358" s="1" t="s">
         <v>736</v>
       </c>
@@ -9360,7 +9359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="359" spans="1:5" hidden="1">
+    <row r="359" spans="1:5">
       <c r="A359" s="1" t="s">
         <v>738</v>
       </c>
@@ -9377,7 +9376,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="360" spans="1:5" hidden="1">
+    <row r="360" spans="1:5">
       <c r="A360" s="1" t="s">
         <v>740</v>
       </c>
@@ -9411,7 +9410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="362" spans="1:5" hidden="1">
+    <row r="362" spans="1:5">
       <c r="A362" s="1" t="s">
         <v>744</v>
       </c>
@@ -9428,7 +9427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="363" spans="1:5" hidden="1">
+    <row r="363" spans="1:5">
       <c r="A363" s="1" t="s">
         <v>746</v>
       </c>
@@ -9445,7 +9444,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="364" spans="1:5" hidden="1">
+    <row r="364" spans="1:5">
       <c r="A364" s="1" t="s">
         <v>748</v>
       </c>
@@ -9462,7 +9461,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="365" spans="1:5" hidden="1">
+    <row r="365" spans="1:5">
       <c r="A365" s="1" t="s">
         <v>750</v>
       </c>
@@ -9479,7 +9478,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="366" spans="1:5" hidden="1">
+    <row r="366" spans="1:5">
       <c r="A366" s="1" t="s">
         <v>752</v>
       </c>
@@ -9496,7 +9495,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="367" spans="1:5" hidden="1">
+    <row r="367" spans="1:5">
       <c r="A367" s="1" t="s">
         <v>754</v>
       </c>
@@ -9513,7 +9512,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="368" spans="1:5" hidden="1">
+    <row r="368" spans="1:5">
       <c r="A368" s="1" t="s">
         <v>756</v>
       </c>
@@ -9530,7 +9529,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="369" spans="1:5" hidden="1">
+    <row r="369" spans="1:5">
       <c r="A369" s="1" t="s">
         <v>758</v>
       </c>
@@ -9538,7 +9537,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="370" spans="1:5" hidden="1">
+    <row r="370" spans="1:5">
       <c r="A370" s="1" t="s">
         <v>760</v>
       </c>
@@ -9555,7 +9554,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="371" spans="1:5" hidden="1">
+    <row r="371" spans="1:5">
       <c r="A371" s="1" t="s">
         <v>762</v>
       </c>
@@ -9572,7 +9571,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="372" spans="1:5" hidden="1">
+    <row r="372" spans="1:5">
       <c r="A372" s="1" t="s">
         <v>764</v>
       </c>
@@ -9589,7 +9588,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="373" spans="1:5" hidden="1">
+    <row r="373" spans="1:5">
       <c r="A373" s="1" t="s">
         <v>766</v>
       </c>
@@ -9606,7 +9605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="374" spans="1:5" hidden="1">
+    <row r="374" spans="1:5">
       <c r="A374" s="1" t="s">
         <v>768</v>
       </c>
@@ -9623,7 +9622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="375" spans="1:5" hidden="1">
+    <row r="375" spans="1:5">
       <c r="A375" s="1" t="s">
         <v>769</v>
       </c>
@@ -9640,7 +9639,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="376" spans="1:5" hidden="1">
+    <row r="376" spans="1:5">
       <c r="A376" s="1" t="s">
         <v>771</v>
       </c>
@@ -9657,7 +9656,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="377" spans="1:5" hidden="1">
+    <row r="377" spans="1:5">
       <c r="A377" s="1" t="s">
         <v>773</v>
       </c>
@@ -9674,7 +9673,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="378" spans="1:5" hidden="1">
+    <row r="378" spans="1:5">
       <c r="A378" s="1" t="s">
         <v>775</v>
       </c>
@@ -9691,7 +9690,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="379" spans="1:5" hidden="1">
+    <row r="379" spans="1:5">
       <c r="A379" s="1" t="s">
         <v>777</v>
       </c>
@@ -9708,7 +9707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="380" spans="1:5" hidden="1">
+    <row r="380" spans="1:5">
       <c r="A380" s="1" t="s">
         <v>779</v>
       </c>
@@ -9725,7 +9724,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="381" spans="1:5" hidden="1">
+    <row r="381" spans="1:5">
       <c r="A381" s="1" t="s">
         <v>781</v>
       </c>
@@ -9742,7 +9741,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="382" spans="1:5" hidden="1">
+    <row r="382" spans="1:5">
       <c r="A382" s="1" t="s">
         <v>783</v>
       </c>
@@ -9759,7 +9758,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="383" spans="1:5" hidden="1">
+    <row r="383" spans="1:5">
       <c r="A383" s="1" t="s">
         <v>785</v>
       </c>
@@ -9776,7 +9775,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="384" spans="1:5" hidden="1">
+    <row r="384" spans="1:5">
       <c r="A384" s="1" t="s">
         <v>787</v>
       </c>
@@ -9793,7 +9792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="385" spans="1:5" hidden="1">
+    <row r="385" spans="1:5">
       <c r="A385" s="1" t="s">
         <v>789</v>
       </c>
@@ -9810,7 +9809,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="386" spans="1:5" hidden="1">
+    <row r="386" spans="1:5">
       <c r="A386" s="1" t="s">
         <v>791</v>
       </c>
@@ -9827,7 +9826,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="387" spans="1:5" hidden="1">
+    <row r="387" spans="1:5">
       <c r="A387" s="1" t="s">
         <v>793</v>
       </c>
@@ -9844,7 +9843,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="388" spans="1:5" hidden="1">
+    <row r="388" spans="1:5">
       <c r="A388" s="1" t="s">
         <v>795</v>
       </c>
@@ -9861,7 +9860,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="389" spans="1:5" hidden="1">
+    <row r="389" spans="1:5">
       <c r="A389" s="1" t="s">
         <v>797</v>
       </c>
@@ -9878,7 +9877,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="390" spans="1:5" hidden="1">
+    <row r="390" spans="1:5">
       <c r="A390" s="1" t="s">
         <v>799</v>
       </c>
@@ -9895,7 +9894,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="391" spans="1:5" hidden="1">
+    <row r="391" spans="1:5">
       <c r="A391" s="1" t="s">
         <v>801</v>
       </c>
@@ -9912,7 +9911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="392" spans="1:5" hidden="1">
+    <row r="392" spans="1:5">
       <c r="A392" s="1" t="s">
         <v>803</v>
       </c>
@@ -9929,7 +9928,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="393" spans="1:5" hidden="1">
+    <row r="393" spans="1:5">
       <c r="A393" s="1" t="s">
         <v>805</v>
       </c>
@@ -9946,7 +9945,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="394" spans="1:5" hidden="1">
+    <row r="394" spans="1:5">
       <c r="A394" s="1" t="s">
         <v>807</v>
       </c>
@@ -9963,7 +9962,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="395" spans="1:5" hidden="1">
+    <row r="395" spans="1:5">
       <c r="A395" s="1" t="s">
         <v>809</v>
       </c>
@@ -9980,7 +9979,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="396" spans="1:5" hidden="1">
+    <row r="396" spans="1:5">
       <c r="A396" s="1" t="s">
         <v>811</v>
       </c>
@@ -9997,7 +9996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="397" spans="1:5" hidden="1">
+    <row r="397" spans="1:5">
       <c r="A397" s="1" t="s">
         <v>813</v>
       </c>
@@ -10014,7 +10013,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="398" spans="1:5" hidden="1">
+    <row r="398" spans="1:5">
       <c r="A398" s="1" t="s">
         <v>815</v>
       </c>
@@ -10031,7 +10030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="399" spans="1:5" hidden="1">
+    <row r="399" spans="1:5">
       <c r="A399" s="1" t="s">
         <v>817</v>
       </c>
@@ -10048,7 +10047,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="400" spans="1:5" hidden="1">
+    <row r="400" spans="1:5">
       <c r="A400" s="1" t="s">
         <v>819</v>
       </c>
@@ -10065,7 +10064,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="401" spans="1:5" hidden="1">
+    <row r="401" spans="1:5">
       <c r="A401" s="1" t="s">
         <v>821</v>
       </c>
@@ -10082,7 +10081,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="402" spans="1:5" hidden="1">
+    <row r="402" spans="1:5">
       <c r="A402" s="1" t="s">
         <v>823</v>
       </c>
@@ -10099,7 +10098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="403" spans="1:5" hidden="1">
+    <row r="403" spans="1:5">
       <c r="A403" s="1" t="s">
         <v>825</v>
       </c>
@@ -10116,7 +10115,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="404" spans="1:5" hidden="1">
+    <row r="404" spans="1:5">
       <c r="A404" s="1" t="s">
         <v>827</v>
       </c>
@@ -10133,7 +10132,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="405" spans="1:5" hidden="1">
+    <row r="405" spans="1:5">
       <c r="A405" s="1" t="s">
         <v>829</v>
       </c>
@@ -10150,7 +10149,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="406" spans="1:5" hidden="1">
+    <row r="406" spans="1:5">
       <c r="A406" s="1" t="s">
         <v>831</v>
       </c>
@@ -10167,7 +10166,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="407" spans="1:5" hidden="1">
+    <row r="407" spans="1:5">
       <c r="A407" s="1" t="s">
         <v>833</v>
       </c>
@@ -10184,7 +10183,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="408" spans="1:5" hidden="1">
+    <row r="408" spans="1:5">
       <c r="A408" s="1" t="s">
         <v>835</v>
       </c>
@@ -10201,7 +10200,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="409" spans="1:5" hidden="1">
+    <row r="409" spans="1:5">
       <c r="A409" s="1" t="s">
         <v>837</v>
       </c>
@@ -10218,7 +10217,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="410" spans="1:5" hidden="1">
+    <row r="410" spans="1:5">
       <c r="A410" s="1" t="s">
         <v>839</v>
       </c>
@@ -10235,7 +10234,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="411" spans="1:5" hidden="1">
+    <row r="411" spans="1:5">
       <c r="A411" s="1" t="s">
         <v>841</v>
       </c>
@@ -10252,7 +10251,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="412" spans="1:5" hidden="1">
+    <row r="412" spans="1:5">
       <c r="A412" s="1" t="s">
         <v>843</v>
       </c>
@@ -10269,7 +10268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="413" spans="1:5" hidden="1">
+    <row r="413" spans="1:5">
       <c r="A413" s="1" t="s">
         <v>845</v>
       </c>
@@ -10286,7 +10285,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="414" spans="1:5" hidden="1">
+    <row r="414" spans="1:5">
       <c r="A414" s="1" t="s">
         <v>847</v>
       </c>
@@ -10303,7 +10302,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="415" spans="1:5" hidden="1">
+    <row r="415" spans="1:5">
       <c r="A415" s="1" t="s">
         <v>849</v>
       </c>
@@ -10320,7 +10319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="416" spans="1:5" hidden="1">
+    <row r="416" spans="1:5">
       <c r="A416" s="1" t="s">
         <v>851</v>
       </c>
@@ -10337,7 +10336,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="417" spans="1:5" hidden="1">
+    <row r="417" spans="1:5">
       <c r="A417" s="1" t="s">
         <v>853</v>
       </c>
@@ -10354,7 +10353,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="418" spans="1:5" hidden="1">
+    <row r="418" spans="1:5">
       <c r="A418" s="1" t="s">
         <v>855</v>
       </c>
@@ -10371,7 +10370,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="419" spans="1:5" hidden="1">
+    <row r="419" spans="1:5">
       <c r="A419" s="1" t="s">
         <v>857</v>
       </c>
@@ -10388,7 +10387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="420" spans="1:5" hidden="1">
+    <row r="420" spans="1:5">
       <c r="A420" s="1" t="s">
         <v>859</v>
       </c>
@@ -10405,7 +10404,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="421" spans="1:5" hidden="1">
+    <row r="421" spans="1:5">
       <c r="A421" s="1" t="s">
         <v>861</v>
       </c>
@@ -10422,7 +10421,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="422" spans="1:5" hidden="1">
+    <row r="422" spans="1:5">
       <c r="A422" s="1" t="s">
         <v>863</v>
       </c>
@@ -10439,7 +10438,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="423" spans="1:5" hidden="1">
+    <row r="423" spans="1:5">
       <c r="A423" s="1" t="s">
         <v>865</v>
       </c>
@@ -10456,7 +10455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="424" spans="1:5" hidden="1">
+    <row r="424" spans="1:5">
       <c r="A424" s="1" t="s">
         <v>867</v>
       </c>
@@ -10473,7 +10472,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="425" spans="1:5" hidden="1">
+    <row r="425" spans="1:5">
       <c r="A425" s="1" t="s">
         <v>869</v>
       </c>
@@ -10490,7 +10489,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="426" spans="1:5" hidden="1">
+    <row r="426" spans="1:5">
       <c r="A426" s="1" t="s">
         <v>871</v>
       </c>
@@ -10507,7 +10506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="427" spans="1:5" hidden="1">
+    <row r="427" spans="1:5">
       <c r="A427" s="1" t="s">
         <v>873</v>
       </c>
@@ -10524,7 +10523,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="428" spans="1:5" hidden="1">
+    <row r="428" spans="1:5">
       <c r="A428" s="1" t="s">
         <v>875</v>
       </c>
@@ -10541,7 +10540,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="429" spans="1:5" hidden="1">
+    <row r="429" spans="1:5">
       <c r="A429" s="1" t="s">
         <v>877</v>
       </c>
@@ -10558,7 +10557,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="430" spans="1:5" hidden="1">
+    <row r="430" spans="1:5">
       <c r="A430" s="1" t="s">
         <v>879</v>
       </c>
@@ -10575,7 +10574,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="431" spans="1:5" hidden="1">
+    <row r="431" spans="1:5">
       <c r="A431" s="1" t="s">
         <v>881</v>
       </c>
@@ -10592,7 +10591,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="432" spans="1:5" hidden="1">
+    <row r="432" spans="1:5">
       <c r="A432" s="1" t="s">
         <v>883</v>
       </c>
@@ -10609,7 +10608,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="433" spans="1:5" hidden="1">
+    <row r="433" spans="1:5">
       <c r="A433" s="1" t="s">
         <v>885</v>
       </c>
@@ -10626,7 +10625,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="434" spans="1:5" hidden="1">
+    <row r="434" spans="1:5">
       <c r="A434" s="1" t="s">
         <v>887</v>
       </c>
@@ -10643,7 +10642,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="435" spans="1:5" hidden="1">
+    <row r="435" spans="1:5">
       <c r="A435" s="1" t="s">
         <v>889</v>
       </c>
@@ -10660,7 +10659,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="436" spans="1:5" hidden="1">
+    <row r="436" spans="1:5">
       <c r="A436" s="1" t="s">
         <v>891</v>
       </c>
@@ -10677,7 +10676,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="437" spans="1:5" hidden="1">
+    <row r="437" spans="1:5">
       <c r="A437" s="1" t="s">
         <v>893</v>
       </c>
@@ -10694,7 +10693,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="438" spans="1:5" hidden="1">
+    <row r="438" spans="1:5">
       <c r="A438" s="1" t="s">
         <v>895</v>
       </c>
@@ -10711,7 +10710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="439" spans="1:5" hidden="1">
+    <row r="439" spans="1:5">
       <c r="A439" s="1" t="s">
         <v>897</v>
       </c>
@@ -10728,7 +10727,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="440" spans="1:5" hidden="1">
+    <row r="440" spans="1:5">
       <c r="A440" s="1" t="s">
         <v>899</v>
       </c>
@@ -10745,7 +10744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="441" spans="1:5" hidden="1">
+    <row r="441" spans="1:5">
       <c r="A441" s="1" t="s">
         <v>901</v>
       </c>
@@ -10762,7 +10761,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="442" spans="1:5" hidden="1">
+    <row r="442" spans="1:5">
       <c r="A442" s="1" t="s">
         <v>903</v>
       </c>
@@ -10779,7 +10778,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="443" spans="1:5" hidden="1">
+    <row r="443" spans="1:5">
       <c r="A443" s="1" t="s">
         <v>905</v>
       </c>
@@ -10796,7 +10795,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="444" spans="1:5" hidden="1">
+    <row r="444" spans="1:5">
       <c r="A444" s="1" t="s">
         <v>907</v>
       </c>
@@ -10813,7 +10812,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="445" spans="1:5" hidden="1">
+    <row r="445" spans="1:5">
       <c r="A445" s="1" t="s">
         <v>909</v>
       </c>
@@ -10830,7 +10829,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="446" spans="1:5" hidden="1">
+    <row r="446" spans="1:5">
       <c r="A446" s="1" t="s">
         <v>911</v>
       </c>
@@ -10847,7 +10846,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="447" spans="1:5" hidden="1">
+    <row r="447" spans="1:5">
       <c r="A447" s="1" t="s">
         <v>913</v>
       </c>
@@ -10864,7 +10863,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="448" spans="1:5" hidden="1">
+    <row r="448" spans="1:5">
       <c r="A448" s="1" t="s">
         <v>915</v>
       </c>
@@ -10881,7 +10880,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="449" spans="1:5" hidden="1">
+    <row r="449" spans="1:5">
       <c r="A449" s="1" t="s">
         <v>917</v>
       </c>
@@ -10898,7 +10897,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="450" spans="1:5" hidden="1">
+    <row r="450" spans="1:5">
       <c r="A450" s="1" t="s">
         <v>919</v>
       </c>
@@ -10915,7 +10914,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="451" spans="1:5" hidden="1">
+    <row r="451" spans="1:5">
       <c r="A451" s="1" t="s">
         <v>921</v>
       </c>
@@ -10932,7 +10931,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="452" spans="1:5" hidden="1">
+    <row r="452" spans="1:5">
       <c r="A452" s="1" t="s">
         <v>923</v>
       </c>
@@ -10949,7 +10948,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="453" spans="1:5" hidden="1">
+    <row r="453" spans="1:5">
       <c r="A453" s="1" t="s">
         <v>925</v>
       </c>
@@ -10966,7 +10965,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="454" spans="1:5" hidden="1">
+    <row r="454" spans="1:5">
       <c r="A454" s="1" t="s">
         <v>927</v>
       </c>
@@ -10983,7 +10982,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="455" spans="1:5" hidden="1">
+    <row r="455" spans="1:5">
       <c r="A455" s="1" t="s">
         <v>929</v>
       </c>
@@ -11000,7 +10999,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="456" spans="1:5" hidden="1">
+    <row r="456" spans="1:5">
       <c r="A456" s="1" t="s">
         <v>931</v>
       </c>
@@ -11017,7 +11016,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="457" spans="1:5" hidden="1">
+    <row r="457" spans="1:5">
       <c r="A457" s="1" t="s">
         <v>933</v>
       </c>
@@ -11035,13 +11034,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E457" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="EM"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:E457" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>